<commit_message>
Commit on Hybrid F/W
</commit_message>
<xml_diff>
--- a/AutoNexus/testData/LoginData.xlsx
+++ b/AutoNexus/testData/LoginData.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>username</t>
   </si>
@@ -27,7 +27,7 @@
     <t>result</t>
   </si>
   <si>
-    <t>Justin@gmal3.1.com</t>
+    <t>Justin@gmal3.1222.com</t>
   </si>
   <si>
     <t>abc</t>
@@ -36,7 +36,13 @@
     <t>Invalid</t>
   </si>
   <si>
+    <t>4asd</t>
+  </si>
+  <si>
     <t>vfedsg2</t>
+  </si>
+  <si>
+    <t>123456</t>
   </si>
   <si>
     <t>Valid</t>
@@ -52,7 +58,7 @@
   <fonts count="4">
     <font>
       <sz val="10.000000"/>
-      <color indexed="64"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
@@ -71,7 +77,7 @@
     <font>
       <sz val="11.000000"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -101,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment readingOrder="0"/>
     </xf>
@@ -115,8 +121,12 @@
     <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf fontId="3" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf fontId="3" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" quotePrefix="1">
       <alignment readingOrder="0"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1" quotePrefix="1">
+      <alignment readingOrder="0"/>
+      <protection hidden="0" locked="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -618,7 +628,7 @@
   </sheetPr>
   <sheetFormatPr defaultColWidth="12.630000000000001" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="20.629999999999999"/>
+    <col bestFit="1" customWidth="1" min="1" max="1" width="21.61328125"/>
     <col customWidth="1" min="2" max="2" width="18.75"/>
   </cols>
   <sheetData>
@@ -634,7 +644,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="s">
+      <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -645,45 +655,45 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="s">
+      <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="4">
-        <v>4</v>
+      <c r="B3" s="4" t="s">
+        <v>6</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2">
-        <v>321</v>
+      <c r="A4" s="2"/>
+      <c r="B4" s="2" t="s">
+        <v>7</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2" t="s">
-        <v>6</v>
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="2">
+        <v>321</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="s">
+      <c r="A6" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="2">
-        <v>12345</v>
+      <c r="B6" s="5" t="s">
+        <v>8</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>